<commit_message>
DATN ho Ca Giay: Excel kiem tra kha nang thoat nuoc cua ranh mai ha luu (Bang 5.6)
Sheet Bang5_6_Ranh: Qtk = C.i.A, Qtn Manning o 75% chieu cao ranh, chieu sau va luu toc khi xa Qtk,
kiem tra bat loi; dung chung so lieu mua, hinh hoc mai voi Bang 5.5.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FZ7RkEfpZxiJWB6royQwfj
</commit_message>
<xml_diff>
--- a/DATN_HoCaGiay/TAI_VE/DongChayTranMai_Bang5_5.xlsx
+++ b/DATN_HoCaGiay/TAI_VE/DongChayTranMai_Bang5_5.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bang5_5" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DoNhay" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BieuDo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bang5_6_Ranh" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="Mua_ngay">SoLieu!$B$6</definedName>
@@ -36,6 +37,15 @@
     <definedName name="tau_cat">SoLieu!$B$34</definedName>
     <definedName name="tau_bui">SoLieu!$B$35</definedName>
     <definedName name="tau_thit">SoLieu!$B$36</definedName>
+    <definedName name="n_BT">SoLieu!$B$40</definedName>
+    <definedName name="Ty_le_sau">SoLieu!$B$41</definedName>
+    <definedName name="K_doc">SoLieu!$B$42</definedName>
+    <definedName name="B_dinh">SoLieu!$B$43</definedName>
+    <definedName name="B_co">SoLieu!$B$44</definedName>
+    <definedName name="D_chan">SoLieu!$B$45</definedName>
+    <definedName name="i_ngang">SoLieu!$B$46</definedName>
+    <definedName name="X_tren">SoLieu!$B$47</definedName>
+    <definedName name="X_duoi">SoLieu!$B$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -150,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -239,6 +249,18 @@
     </xf>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -907,7 +929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -917,7 +939,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DÒNG CHẢY TRÀN TRÊN MÁI HẠ LƯU KHI MƯA – HIỆU QUẢ CHỐNG XÓI CỦA VIỆC CHIA Ô MÁI (Bảng 5.5)</t>
+          <t>DÒNG CHẢY TRÀN TRÊN MÁI HẠ LƯU KHI MƯA – CHIA Ô MÁI VÀ KIỂM TRA RÃNH THOÁT NƯỚC (mục 5.4.1, 5.4.2)</t>
         </is>
       </c>
     </row>
@@ -1086,6 +1108,65 @@
       <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Chiều dài cả mái trên tính đúng là 34,3 m; bảng làm tròn 34 m như thuyết minh (τ chênh 0,04 Pa).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>5. Kiểm tra khả năng thoát nước của rãnh (sheet Bang5_6_Ranh)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="3" t="inlineStr"/>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Qtk = C·i·A      – lưu lượng thiết kế: phương pháp cường độ giới hạn, A – diện tích hứng nước (hình chiếu ngang).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="3" t="inlineStr"/>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Qtn = (1/n)·ω·R^(2/3)·√S – khả năng thoát (Manning), nước sâu h = 0,75·H; ω = b·h; χ = b + 2h; R = ω/χ; v = Qtn/ω.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Diện tích hứng nước: rãnh dọc – khoảng cách rãnh 40 m × (bề rộng đỉnh + hình chiếu ngang mái trên); rãnh ngang trên cơ – 40 m × (bề rộng cơ + dải chân mái trên); rãnh xiên – một ô 4 × 4 m; rãnh ngang đỉnh – 40 m × bề rộng đỉnh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Độ dốc S: rãnh dọc chạy theo đường dốc nhất S = sinβ; rãnh xiên lệch 45° trên mặt mái S = sinβ/√2; rãnh ngang (đỉnh, cơ) S = 0,003.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Bảng b) tính chiều sâu và lưu tốc khi rãnh xả đúng Qtk (lặp 5 lần công thức Manning); bảng c) kiểm tra khi nước dồn nhiều hơn giả thiết – vẫn đạt.</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1660,6 +1741,201 @@
           <t>Khi cỏ đã phủ kín, mái chịu được ứng suất tiếp lớn hơn nhiều lần</t>
         </is>
       </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>E. RÃNH THOÁT NƯỚC MÁI (Bảng 5.6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Thông số</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Giá trị</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Đơn vị</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>Ghi chú, nguồn</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>Hệ số nhám rãnh bê tông n</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>Bê tông</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>Chiều sâu nước tính khả năng thoát / chiều cao rãnh</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>Chừa 25% chiều cao an toàn</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>Khoảng cách rãnh dọc</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>TCVN 8216:2018 điều 10.3.4.6: 25 ÷ 50 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>Bề rộng đỉnh đập</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>Dốc ngang về hạ lưu, nước qua khe gờ chắn bánh vào rãnh ngang đỉnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>Bề rộng cơ hạ lưu</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>Dải chân mái trên chảy vào rãnh cơ</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>Giả thiết (khớp diện tích 680 m² của Bảng 5.6); xem bảng c) kiểm tra bất lợi</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>Độ dốc dọc rãnh ngang (đỉnh, cơ)</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>Hình chiếu ngang đoạn mái trên</t>
+        </is>
+      </c>
+      <c r="B47" s="17">
+        <f>m_tren*(Z_dinh-Z_co)</f>
+        <v/>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D47" s="10" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>Hình chiếu ngang đoạn mái dưới</t>
+        </is>
+      </c>
+      <c r="B48" s="17">
+        <f>m_duoi*(Z_co-Z_ltr)</f>
+        <v/>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.4" right="0.4" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3555,4 +3831,813 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00EB6834"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:O26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>BẢNG 5.6 – KIỂM TRA KHẢ NĂNG THOÁT NƯỚC CÁC LOẠI RÃNH MÁI HẠ LƯU</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Qtk = C·i·A;  Qtn = (1/n)·ω·R^(2/3)·√S với chiều sâu nước h = 0,75·H;  ω = b·h;  χ = b + 2h;  R = ω/χ;  v = Qtn/ω. Số liệu ở sheet SoLieu (mục A, B, C, E).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>a) Khả năng thoát nước (cột in đậm là các cột của Bảng 5.6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Loại rãnh</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>b (m)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>H (m)</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>A (m²)</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Cách lấy diện tích hứng nước A</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Qtk = C·i·A (m³/s)</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Độ dốc S</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>h = 0,75·H (m)</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>ω = b·h (m²)</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>χ = b + 2h (m)</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>R = ω/χ (m)</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Qtn (m³/s)</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>v = Qtn/ω (m/s)</t>
+        </is>
+      </c>
+      <c r="N5" s="6" t="inlineStr">
+        <is>
+          <t>Qtn / Qtk (lần)</t>
+        </is>
+      </c>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>Đánh giá</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>Rãnh dọc 40 × 40 cm (theo mái, @ 40 m)</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D6" s="33">
+        <f>K_doc*(B_dinh+X_tren)</f>
+        <v/>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>40 m × (đỉnh 5 m + hình chiếu mái trên)</t>
+        </is>
+      </c>
+      <c r="F6" s="16">
+        <f>HS_C*i_ms*D6</f>
+        <v/>
+      </c>
+      <c r="G6" s="34">
+        <f>sin_tren</f>
+        <v/>
+      </c>
+      <c r="H6" s="32">
+        <f>Ty_le_sau*C6</f>
+        <v/>
+      </c>
+      <c r="I6" s="35">
+        <f>B6*H6</f>
+        <v/>
+      </c>
+      <c r="J6" s="32">
+        <f>B6+2*H6</f>
+        <v/>
+      </c>
+      <c r="K6" s="35">
+        <f>I6/J6</f>
+        <v/>
+      </c>
+      <c r="L6" s="34">
+        <f>I6*K6^(2/3)*SQRT(G6)/n_BT</f>
+        <v/>
+      </c>
+      <c r="M6" s="17">
+        <f>L6/I6</f>
+        <v/>
+      </c>
+      <c r="N6" s="24">
+        <f>L6/F6</f>
+        <v/>
+      </c>
+      <c r="O6" s="31">
+        <f>IF(L6&gt;=F6,"Đạt","Không đạt")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>Rãnh ngang trên cơ 40 × 40 cm</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D7" s="33">
+        <f>K_doc*(B_co+D_chan)</f>
+        <v/>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>40 m × (cơ 14 m + dải chân mái 3 m)</t>
+        </is>
+      </c>
+      <c r="F7" s="16">
+        <f>HS_C*i_ms*D7</f>
+        <v/>
+      </c>
+      <c r="G7" s="34">
+        <f>i_ngang</f>
+        <v/>
+      </c>
+      <c r="H7" s="32">
+        <f>Ty_le_sau*C7</f>
+        <v/>
+      </c>
+      <c r="I7" s="35">
+        <f>B7*H7</f>
+        <v/>
+      </c>
+      <c r="J7" s="32">
+        <f>B7+2*H7</f>
+        <v/>
+      </c>
+      <c r="K7" s="35">
+        <f>I7/J7</f>
+        <v/>
+      </c>
+      <c r="L7" s="34">
+        <f>I7*K7^(2/3)*SQRT(G7)/n_BT</f>
+        <v/>
+      </c>
+      <c r="M7" s="17">
+        <f>L7/I7</f>
+        <v/>
+      </c>
+      <c r="N7" s="24">
+        <f>L7/F7</f>
+        <v/>
+      </c>
+      <c r="O7" s="31">
+        <f>IF(L7&gt;=F7,"Đạt","Không đạt")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>Rãnh xiên 20 × 20 cm (ô 4 × 4 m)</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D8" s="33">
+        <f>a_o^2</f>
+        <v/>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Một ô 4 × 4 m</t>
+        </is>
+      </c>
+      <c r="F8" s="16">
+        <f>HS_C*i_ms*D8</f>
+        <v/>
+      </c>
+      <c r="G8" s="34">
+        <f>sin_tren/SQRT(2)</f>
+        <v/>
+      </c>
+      <c r="H8" s="32">
+        <f>Ty_le_sau*C8</f>
+        <v/>
+      </c>
+      <c r="I8" s="35">
+        <f>B8*H8</f>
+        <v/>
+      </c>
+      <c r="J8" s="32">
+        <f>B8+2*H8</f>
+        <v/>
+      </c>
+      <c r="K8" s="35">
+        <f>I8/J8</f>
+        <v/>
+      </c>
+      <c r="L8" s="34">
+        <f>I8*K8^(2/3)*SQRT(G8)/n_BT</f>
+        <v/>
+      </c>
+      <c r="M8" s="17">
+        <f>L8/I8</f>
+        <v/>
+      </c>
+      <c r="N8" s="24">
+        <f>L8/F8</f>
+        <v/>
+      </c>
+      <c r="O8" s="31">
+        <f>IF(L8&gt;=F8,"Đạt","Không đạt")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>Rãnh ngang đỉnh 20 × 20 cm</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D9" s="33">
+        <f>K_doc*B_dinh</f>
+        <v/>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>40 m × đỉnh 5 m</t>
+        </is>
+      </c>
+      <c r="F9" s="16">
+        <f>HS_C*i_ms*D9</f>
+        <v/>
+      </c>
+      <c r="G9" s="34">
+        <f>i_ngang</f>
+        <v/>
+      </c>
+      <c r="H9" s="32">
+        <f>Ty_le_sau*C9</f>
+        <v/>
+      </c>
+      <c r="I9" s="35">
+        <f>B9*H9</f>
+        <v/>
+      </c>
+      <c r="J9" s="32">
+        <f>B9+2*H9</f>
+        <v/>
+      </c>
+      <c r="K9" s="35">
+        <f>I9/J9</f>
+        <v/>
+      </c>
+      <c r="L9" s="34">
+        <f>I9*K9^(2/3)*SQRT(G9)/n_BT</f>
+        <v/>
+      </c>
+      <c r="M9" s="17">
+        <f>L9/I9</f>
+        <v/>
+      </c>
+      <c r="N9" s="24">
+        <f>L9/F9</f>
+        <v/>
+      </c>
+      <c r="O9" s="31">
+        <f>IF(L9&gt;=F9,"Đạt","Không đạt")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>b) Chiều sâu và lưu tốc khi rãnh xả đúng Qtk – giải lặp công thức Manning: h = (Qtk·n/√S)^0,6·(b + 2h)^0,4 / b</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Loại rãnh</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Qtk (m³/s)</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>h₀ (m)</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>h₁ (m)</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>h₂ (m)</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>h₃ (m)</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>h₄ (m)</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>h (cm)</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>v (m/s)</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>h / H (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="26">
+        <f>A6</f>
+        <v/>
+      </c>
+      <c r="B14" s="35">
+        <f>F6</f>
+        <v/>
+      </c>
+      <c r="C14" s="35">
+        <f>(B14*n_BT/(B6*SQRT(G6)))^0.6</f>
+        <v/>
+      </c>
+      <c r="D14" s="35">
+        <f>(B14*n_BT/SQRT(G6))^0.6*(B6+2*C14)^0.4/B6</f>
+        <v/>
+      </c>
+      <c r="E14" s="35">
+        <f>(B14*n_BT/SQRT(G6))^0.6*(B6+2*D14)^0.4/B6</f>
+        <v/>
+      </c>
+      <c r="F14" s="35">
+        <f>(B14*n_BT/SQRT(G6))^0.6*(B6+2*E14)^0.4/B6</f>
+        <v/>
+      </c>
+      <c r="G14" s="35">
+        <f>(B14*n_BT/SQRT(G6))^0.6*(B6+2*F14)^0.4/B6</f>
+        <v/>
+      </c>
+      <c r="H14" s="12">
+        <f>100*G14</f>
+        <v/>
+      </c>
+      <c r="I14" s="17">
+        <f>B14/(B6*G14)</f>
+        <v/>
+      </c>
+      <c r="J14" s="24">
+        <f>100*G14/C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="26">
+        <f>A7</f>
+        <v/>
+      </c>
+      <c r="B15" s="35">
+        <f>F7</f>
+        <v/>
+      </c>
+      <c r="C15" s="35">
+        <f>(B15*n_BT/(B7*SQRT(G7)))^0.6</f>
+        <v/>
+      </c>
+      <c r="D15" s="35">
+        <f>(B15*n_BT/SQRT(G7))^0.6*(B7+2*C15)^0.4/B7</f>
+        <v/>
+      </c>
+      <c r="E15" s="35">
+        <f>(B15*n_BT/SQRT(G7))^0.6*(B7+2*D15)^0.4/B7</f>
+        <v/>
+      </c>
+      <c r="F15" s="35">
+        <f>(B15*n_BT/SQRT(G7))^0.6*(B7+2*E15)^0.4/B7</f>
+        <v/>
+      </c>
+      <c r="G15" s="35">
+        <f>(B15*n_BT/SQRT(G7))^0.6*(B7+2*F15)^0.4/B7</f>
+        <v/>
+      </c>
+      <c r="H15" s="12">
+        <f>100*G15</f>
+        <v/>
+      </c>
+      <c r="I15" s="17">
+        <f>B15/(B7*G15)</f>
+        <v/>
+      </c>
+      <c r="J15" s="24">
+        <f>100*G15/C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="26">
+        <f>A8</f>
+        <v/>
+      </c>
+      <c r="B16" s="35">
+        <f>F8</f>
+        <v/>
+      </c>
+      <c r="C16" s="35">
+        <f>(B16*n_BT/(B8*SQRT(G8)))^0.6</f>
+        <v/>
+      </c>
+      <c r="D16" s="35">
+        <f>(B16*n_BT/SQRT(G8))^0.6*(B8+2*C16)^0.4/B8</f>
+        <v/>
+      </c>
+      <c r="E16" s="35">
+        <f>(B16*n_BT/SQRT(G8))^0.6*(B8+2*D16)^0.4/B8</f>
+        <v/>
+      </c>
+      <c r="F16" s="35">
+        <f>(B16*n_BT/SQRT(G8))^0.6*(B8+2*E16)^0.4/B8</f>
+        <v/>
+      </c>
+      <c r="G16" s="35">
+        <f>(B16*n_BT/SQRT(G8))^0.6*(B8+2*F16)^0.4/B8</f>
+        <v/>
+      </c>
+      <c r="H16" s="12">
+        <f>100*G16</f>
+        <v/>
+      </c>
+      <c r="I16" s="17">
+        <f>B16/(B8*G16)</f>
+        <v/>
+      </c>
+      <c r="J16" s="24">
+        <f>100*G16/C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="26">
+        <f>A9</f>
+        <v/>
+      </c>
+      <c r="B17" s="35">
+        <f>F9</f>
+        <v/>
+      </c>
+      <c r="C17" s="35">
+        <f>(B17*n_BT/(B9*SQRT(G9)))^0.6</f>
+        <v/>
+      </c>
+      <c r="D17" s="35">
+        <f>(B17*n_BT/SQRT(G9))^0.6*(B9+2*C17)^0.4/B9</f>
+        <v/>
+      </c>
+      <c r="E17" s="35">
+        <f>(B17*n_BT/SQRT(G9))^0.6*(B9+2*D17)^0.4/B9</f>
+        <v/>
+      </c>
+      <c r="F17" s="35">
+        <f>(B17*n_BT/SQRT(G9))^0.6*(B9+2*E17)^0.4/B9</f>
+        <v/>
+      </c>
+      <c r="G17" s="35">
+        <f>(B17*n_BT/SQRT(G9))^0.6*(B9+2*F17)^0.4/B9</f>
+        <v/>
+      </c>
+      <c r="H17" s="12">
+        <f>100*G17</f>
+        <v/>
+      </c>
+      <c r="I17" s="17">
+        <f>B17/(B9*G17)</f>
+        <v/>
+      </c>
+      <c r="J17" s="24">
+        <f>100*G17/C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>c) Kiểm tra bất lợi – nước dồn nhiều hơn giả thiết diện tích hứng nước ở bảng a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Trường hợp</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>b (m)</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>H (m)</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>A (m²)</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Cách lấy diện tích hứng nước A</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Qtk (m³/s)</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Độ dốc S</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>Qtn (m³/s)</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>Qtn / Qtk (lần)</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>Đánh giá</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>Rãnh dọc đoạn dưới cơ (m = 3,5)</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C21" s="11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D21" s="33">
+        <f>K_doc*(B_dinh+X_tren+B_co+X_duoi)</f>
+        <v/>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>Nhận nước đỉnh, mái trên, cơ và mái dưới</t>
+        </is>
+      </c>
+      <c r="F21" s="16">
+        <f>HS_C*i_ms*D21</f>
+        <v/>
+      </c>
+      <c r="G21" s="32">
+        <f>sin_duoi</f>
+        <v/>
+      </c>
+      <c r="H21" s="34">
+        <f>(B21*Ty_le_sau*C21)*((B21*Ty_le_sau*C21)/(B21+2*Ty_le_sau*C21))^(2/3)*SQRT(G21)/n_BT</f>
+        <v/>
+      </c>
+      <c r="I21" s="23">
+        <f>H21/F21</f>
+        <v/>
+      </c>
+      <c r="J21" s="31">
+        <f>IF(H21&gt;=F21,"Đạt","Không đạt")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>Rãnh ngang trên cơ nhận cả nước mái trên</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C22" s="11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D22" s="33">
+        <f>K_doc*(B_dinh+X_tren+B_co)</f>
+        <v/>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>Như rãnh dọc + cả mặt cơ</t>
+        </is>
+      </c>
+      <c r="F22" s="16">
+        <f>HS_C*i_ms*D22</f>
+        <v/>
+      </c>
+      <c r="G22" s="32">
+        <f>i_ngang</f>
+        <v/>
+      </c>
+      <c r="H22" s="34">
+        <f>(B22*Ty_le_sau*C22)*((B22*Ty_le_sau*C22)/(B22+2*Ty_le_sau*C22))^(2/3)*SQRT(G22)/n_BT</f>
+        <v/>
+      </c>
+      <c r="I22" s="23">
+        <f>H22/F22</f>
+        <v/>
+      </c>
+      <c r="J22" s="31">
+        <f>IF(H22&gt;=F22,"Đạt","Không đạt")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>Rãnh xiên nhận nửa khoang mái trên</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D23" s="33">
+        <f>K_doc/2*X_tren</f>
+        <v/>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>20 m × hình chiếu mái trên</t>
+        </is>
+      </c>
+      <c r="F23" s="16">
+        <f>HS_C*i_ms*D23</f>
+        <v/>
+      </c>
+      <c r="G23" s="32">
+        <f>sin_tren/SQRT(2)</f>
+        <v/>
+      </c>
+      <c r="H23" s="34">
+        <f>(B23*Ty_le_sau*C23)*((B23*Ty_le_sau*C23)/(B23+2*Ty_le_sau*C23))^(2/3)*SQRT(G23)/n_BT</f>
+        <v/>
+      </c>
+      <c r="I23" s="23">
+        <f>H23/F23</f>
+        <v/>
+      </c>
+      <c r="J23" s="31">
+        <f>IF(H23&gt;=F23,"Đạt","Không đạt")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="36" t="inlineStr">
+        <is>
+          <t>Ghi chú: v ở bảng a) là lưu tốc khi nước sâu 75% chiều cao rãnh; khi xả đúng Qtk (bảng b) rãnh dọc chỉ ngập khoảng 2,5 cm nhưng lưu tốc ≈ 2,9 m/s – rãnh phải bằng bê tông liền khối, có gờ tiêu năng ở chỗ nối với cơ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="36" t="inlineStr">
+        <is>
+          <t>So với Bảng 5.6 trong thuyết minh: A rãnh dọc 1.460 m² = 40 × (5 + 31,5) ứng với đỉnh +78,50; với đỉnh sau sửa chữa +78,85 là 1.502 m² (Qtk 0,0288 m³/s). Rãnh xiên: bảng cũ lấy độ dốc ≈ 0,24 (= tanβ/√2); theo phương dọc rãnh là sinβ/√2 = 0,224 nên Qtn 0,145 m³/s, v 4,83 m/s (bảng cũ 0,149; 4,96). Kết luận không đổi.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A25:O25"/>
+    <mergeCell ref="A26:O26"/>
+  </mergeCells>
+  <pageMargins left="0.4" right="0.4" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>